<commit_message>
Agregué argumentos de ejecución
</commit_message>
<xml_diff>
--- a/app/src/main/java/tps/tp1/salida/reporte.Xlsx
+++ b/app/src/main/java/tps/tp1/salida/reporte.Xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
   <si>
     <t>Padron</t>
   </si>
@@ -38,19 +38,16 @@
     <t>CON_DEUDA</t>
   </si>
   <si>
+    <t>Elena Sosa</t>
+  </si>
+  <si>
     <t>Ana Gomez</t>
   </si>
   <si>
     <t>Diego Ruiz</t>
   </si>
   <si>
-    <t>Elena Sosa</t>
-  </si>
-  <si>
     <t>Carla Nunez</t>
-  </si>
-  <si>
-    <t>AL_DIA</t>
   </si>
 </sst>
 </file>
@@ -146,10 +143,10 @@
         <v>4.0</v>
       </c>
       <c r="D2" t="n" s="0">
-        <v>24.0</v>
+        <v>157.0</v>
       </c>
       <c r="E2" t="n" s="0">
-        <v>3600.0</v>
+        <v>4800.0</v>
       </c>
       <c r="F2" t="s" s="0">
         <v>7</v>
@@ -157,19 +154,19 @@
     </row>
     <row r="3">
       <c r="A3" t="n" s="0">
-        <v>41234.0</v>
+        <v>43310.0</v>
       </c>
       <c r="B3" t="s" s="0">
         <v>8</v>
       </c>
       <c r="C3" t="n" s="0">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="D3" t="n" s="0">
-        <v>23.0</v>
+        <v>143.0</v>
       </c>
       <c r="E3" t="n" s="0">
-        <v>3450.0</v>
+        <v>4500.0</v>
       </c>
       <c r="F3" t="s" s="0">
         <v>7</v>
@@ -177,19 +174,19 @@
     </row>
     <row r="4">
       <c r="A4" t="n" s="0">
-        <v>40555.0</v>
+        <v>41234.0</v>
       </c>
       <c r="B4" t="s" s="0">
         <v>9</v>
       </c>
       <c r="C4" t="n" s="0">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="D4" t="n" s="0">
-        <v>42.0</v>
+        <v>156.0</v>
       </c>
       <c r="E4" t="n" s="0">
-        <v>3300.0</v>
+        <v>3600.0</v>
       </c>
       <c r="F4" t="s" s="0">
         <v>7</v>
@@ -197,7 +194,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n" s="0">
-        <v>43310.0</v>
+        <v>40555.0</v>
       </c>
       <c r="B5" t="s" s="0">
         <v>10</v>
@@ -206,10 +203,10 @@
         <v>3.0</v>
       </c>
       <c r="D5" t="n" s="0">
-        <v>10.0</v>
+        <v>175.0</v>
       </c>
       <c r="E5" t="n" s="0">
-        <v>1500.0</v>
+        <v>3300.0</v>
       </c>
       <c r="F5" t="s" s="0">
         <v>7</v>
@@ -226,13 +223,13 @@
         <v>4.0</v>
       </c>
       <c r="D6" t="n" s="0">
-        <v>0.0</v>
+        <v>126.0</v>
       </c>
       <c r="E6" t="n" s="0">
-        <v>0.0</v>
+        <v>3000.0</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bugs menores en exportadoXlsx y txt
</commit_message>
<xml_diff>
--- a/app/src/main/java/tps/tp1/salida/reporte.Xlsx
+++ b/app/src/main/java/tps/tp1/salida/reporte.Xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
   <si>
     <t>Padron</t>
   </si>
@@ -38,16 +38,19 @@
     <t>CON_DEUDA</t>
   </si>
   <si>
+    <t>Ana Gomez</t>
+  </si>
+  <si>
+    <t>Diego Ruiz</t>
+  </si>
+  <si>
     <t>Elena Sosa</t>
   </si>
   <si>
-    <t>Ana Gomez</t>
-  </si>
-  <si>
-    <t>Diego Ruiz</t>
-  </si>
-  <si>
     <t>Carla Nunez</t>
+  </si>
+  <si>
+    <t>AL_DIA</t>
   </si>
 </sst>
 </file>
@@ -143,10 +146,10 @@
         <v>4.0</v>
       </c>
       <c r="D2" t="n" s="0">
-        <v>157.0</v>
+        <v>24.0</v>
       </c>
       <c r="E2" t="n" s="0">
-        <v>4800.0</v>
+        <v>3600.0</v>
       </c>
       <c r="F2" t="s" s="0">
         <v>7</v>
@@ -154,19 +157,19 @@
     </row>
     <row r="3">
       <c r="A3" t="n" s="0">
-        <v>43310.0</v>
+        <v>41234.0</v>
       </c>
       <c r="B3" t="s" s="0">
         <v>8</v>
       </c>
       <c r="C3" t="n" s="0">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="D3" t="n" s="0">
-        <v>143.0</v>
+        <v>23.0</v>
       </c>
       <c r="E3" t="n" s="0">
-        <v>4500.0</v>
+        <v>3450.0</v>
       </c>
       <c r="F3" t="s" s="0">
         <v>7</v>
@@ -174,19 +177,19 @@
     </row>
     <row r="4">
       <c r="A4" t="n" s="0">
-        <v>41234.0</v>
+        <v>40555.0</v>
       </c>
       <c r="B4" t="s" s="0">
         <v>9</v>
       </c>
       <c r="C4" t="n" s="0">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="D4" t="n" s="0">
-        <v>156.0</v>
+        <v>42.0</v>
       </c>
       <c r="E4" t="n" s="0">
-        <v>3600.0</v>
+        <v>3300.0</v>
       </c>
       <c r="F4" t="s" s="0">
         <v>7</v>
@@ -194,7 +197,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n" s="0">
-        <v>40555.0</v>
+        <v>43310.0</v>
       </c>
       <c r="B5" t="s" s="0">
         <v>10</v>
@@ -203,10 +206,10 @@
         <v>3.0</v>
       </c>
       <c r="D5" t="n" s="0">
-        <v>175.0</v>
+        <v>10.0</v>
       </c>
       <c r="E5" t="n" s="0">
-        <v>3300.0</v>
+        <v>1500.0</v>
       </c>
       <c r="F5" t="s" s="0">
         <v>7</v>
@@ -223,13 +226,13 @@
         <v>4.0</v>
       </c>
       <c r="D6" t="n" s="0">
-        <v>126.0</v>
+        <v>0.0</v>
       </c>
       <c r="E6" t="n" s="0">
-        <v>3000.0</v>
+        <v>0.0</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>